<commit_message>
Julia changes for ZF
</commit_message>
<xml_diff>
--- a/example_output/pySODA_results_example_image.xlsx
+++ b/example_output/pySODA_results_example_image.xlsx
@@ -409,13 +409,13 @@
         <v>353</v>
       </c>
       <c r="E2">
-        <v>0.08522276569931808</v>
+        <v>0.08522276569931804</v>
       </c>
       <c r="F2">
-        <v>0.1686622356406108</v>
+        <v>0.1686622356406107</v>
       </c>
       <c r="G2">
-        <v>9.604942948202932</v>
+        <v>9.604942948202936</v>
       </c>
     </row>
   </sheetData>

</xml_diff>